<commit_message>
renamed mode = "P" to "W" and "P2" to "P"; fixed error in converting C_xi^P to dB
</commit_message>
<xml_diff>
--- a/results/NDDHO N_xi Data [T_xi_len_s=25, Qs=[20, 40, 60, 80, 100], int 25ms, bw=10p max, kaiser, df=50hz, rip=100db, crop=200hz, tau=500ms, hop_psd=250ms, nfft=None, win=hann].xlsx
+++ b/results/NDDHO N_xi Data [T_xi_len_s=25, Qs=[20, 40, 60, 80, 100], int 25ms, bw=10p max, kaiser, df=50hz, rip=100db, crop=200hz, tau=500ms, hop_psd=250ms, nfft=None, win=hann].xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -638,7 +638,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -754,7 +754,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -870,7 +870,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -986,7 +986,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -4698,7 +4698,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -6090,7 +6090,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -6206,7 +6206,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -6438,7 +6438,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -6554,7 +6554,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -6670,7 +6670,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -7018,7 +7018,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -7134,7 +7134,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -7482,7 +7482,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -7598,7 +7598,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -7946,7 +7946,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -8062,7 +8062,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -8294,7 +8294,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -8410,7 +8410,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E138" t="n">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E142" t="n">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E144" t="n">
@@ -8874,7 +8874,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E146" t="n">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E148" t="n">
@@ -9106,7 +9106,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -9338,7 +9338,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -9570,7 +9570,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -9686,7 +9686,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -9918,7 +9918,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E164" t="n">
@@ -10034,7 +10034,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -10150,7 +10150,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -10266,7 +10266,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -10382,7 +10382,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E172" t="n">
@@ -10498,7 +10498,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E176" t="n">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E178" t="n">
@@ -10846,7 +10846,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E180" t="n">
@@ -10962,7 +10962,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E182" t="n">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E184" t="n">
@@ -11194,7 +11194,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E186" t="n">
@@ -11310,7 +11310,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -11426,7 +11426,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -11542,7 +11542,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E194" t="n">
@@ -11774,7 +11774,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E196" t="n">
@@ -11890,7 +11890,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -12006,7 +12006,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -12122,7 +12122,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E202" t="n">
@@ -12238,7 +12238,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E204" t="n">
@@ -12354,7 +12354,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E206" t="n">
@@ -12470,7 +12470,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E208" t="n">
@@ -12586,7 +12586,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E210" t="n">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E212" t="n">
@@ -12818,7 +12818,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E214" t="n">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E216" t="n">
@@ -13050,7 +13050,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E218" t="n">
@@ -13166,7 +13166,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E220" t="n">
@@ -13282,7 +13282,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E222" t="n">
@@ -13398,7 +13398,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E224" t="n">
@@ -13514,7 +13514,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E226" t="n">
@@ -13630,7 +13630,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E228" t="n">
@@ -13746,7 +13746,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E230" t="n">
@@ -13862,7 +13862,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E232" t="n">
@@ -13978,7 +13978,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E234" t="n">
@@ -14094,7 +14094,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E236" t="n">
@@ -14210,7 +14210,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E238" t="n">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E240" t="n">
@@ -14442,7 +14442,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E242" t="n">
@@ -14558,7 +14558,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E244" t="n">
@@ -14674,7 +14674,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E246" t="n">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E248" t="n">
@@ -14906,7 +14906,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E250" t="n">
@@ -15022,7 +15022,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E252" t="n">
@@ -15138,7 +15138,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E254" t="n">
@@ -15254,7 +15254,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E256" t="n">
@@ -15370,7 +15370,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E258" t="n">
@@ -15486,7 +15486,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E260" t="n">
@@ -15602,7 +15602,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E262" t="n">
@@ -15718,7 +15718,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E264" t="n">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E266" t="n">
@@ -15950,7 +15950,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E268" t="n">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E270" t="n">
@@ -16182,7 +16182,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E272" t="n">
@@ -16298,7 +16298,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E274" t="n">
@@ -16414,7 +16414,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E276" t="n">
@@ -16530,7 +16530,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E278" t="n">
@@ -16646,7 +16646,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E280" t="n">
@@ -16762,7 +16762,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E282" t="n">
@@ -16878,7 +16878,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E284" t="n">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E286" t="n">
@@ -17110,7 +17110,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E288" t="n">
@@ -17226,7 +17226,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E290" t="n">
@@ -17342,7 +17342,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E292" t="n">
@@ -17458,7 +17458,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E294" t="n">
@@ -17574,7 +17574,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E296" t="n">
@@ -17690,7 +17690,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E298" t="n">
@@ -17806,7 +17806,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E300" t="n">

</xml_diff>